<commit_message>
creacion del proceso etl del sa
</commit_message>
<xml_diff>
--- a/DW/Diseño DW.xlsx
+++ b/DW/Diseño DW.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uhispano-my.sharepoint.com/personal/anthony_villalobos0872_uhispano_ac_cr/Documents/Universidad/VII Cuatri/BD/Proyecto/DW/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="54" documentId="8_{7B331317-0294-4D6A-A2AB-5A9A270C473C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{31B4CA53-E7D8-4A4A-9007-2156E02BC628}"/>
+  <xr:revisionPtr revIDLastSave="69" documentId="8_{7B331317-0294-4D6A-A2AB-5A9A270C473C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5FB1B47D-F34D-4C9A-9471-8FE4B9E5B6C6}"/>
   <bookViews>
-    <workbookView xWindow="29760" yWindow="960" windowWidth="21600" windowHeight="11235" activeTab="2" xr2:uid="{4FD1E55B-BC30-4A39-93B9-D1E5AFCC1232}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{4FD1E55B-BC30-4A39-93B9-D1E5AFCC1232}"/>
   </bookViews>
   <sheets>
     <sheet name="ER" sheetId="1" r:id="rId1"/>
@@ -1105,7 +1105,7 @@
   </inkml:definitions>
   <inkml:trace contextRef="#ctx0" brushRef="#br0">189 366 24575,'-1'0'0,"0"1"0,0-1 0,1 0 0,-1 1 0,0-1 0,0 0 0,0 1 0,0-1 0,0 1 0,0 0 0,1-1 0,-1 1 0,0 0 0,1-1 0,-1 1 0,0 0 0,1 0 0,-1 0 0,1-1 0,-1 1 0,1 0 0,-1 0 0,1 0 0,0 0 0,0 0 0,-1 0 0,1 1 0,-5 32 0,4-31 0,-6 110-329,-5 41-187,0 33 59,11-134 203,-2 0 1,-2 0-1,-21 87 0,11-89 384,-8 19 417,4 2 0,3 0-1,-10 101 1,29-593-547,-5 220 0,4 171 0,1 1 0,6-29 0,-3 28 0,2-54 0,-8 42-1365,0 22-5461</inkml:trace>
   <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="556.39">12 267 24575,'11'-1'0,"1"0"0,-1-1 0,0 0 0,13-5 0,40-5 0,-29 10 0,13-1 0,60-10 0,-70 5 0,-1-1 0,-1-2 0,0-2 0,65-32 0,163-69 0,-250 108 0,-6 2 0,-1 1 0,0 1 0,1-1 0,0 1 0,11-1 0,-18 3 0,0 0 0,1 0 0,-1 0 0,1 0 0,-1 0 0,1 0 0,-1 0 0,0 1 0,1-1 0,-1 0 0,0 1 0,1 0 0,-1-1 0,0 1 0,0 0 0,1-1 0,-1 1 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,-1 1 0,1-1 0,0 0 0,-1 0 0,1 1 0,-1-1 0,1 0 0,-1 1 0,0-1 0,1 3 0,2 23 0,-1-1 0,-1 1 0,-5 52 0,-1-1 0,4-62 0,0-1 0,-2 0 0,0 0 0,0 0 0,-2-1 0,0 1 0,0-1 0,-2 0 0,0 0 0,-10 15 0,-2-1 0,-1-1 0,-1-1 0,-39 37 0,57-60 5,-1 0 0,0-1 0,1 0 0,-1 0-1,-1 0 1,1 0 0,0-1 0,0 1 0,-1-1 0,1 0 0,0 0-1,-1-1 1,1 0 0,-1 1 0,-6-2 0,-28 6-1448,22 0-5383</inkml:trace>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="1206.59">1018 1225 24575,'1'-10'0,"1"-1"0,0 1 0,0 0 0,7-17 0,1-9 0,-9 31 0,10-44 0,24-65 0,-33 109 0,1 1 0,-1 0 0,1-1 0,0 1 0,0 0 0,0 0 0,1 1 0,0-1 0,-1 1 0,1-1 0,1 1 0,-1 0 0,0 1 0,5-3 0,11-5 0,1 2 0,22-8 0,24-9 0,-27 5-455,0 2 0,68-19 0,-90 32-6371</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="1206.58">1018 1225 24575,'1'-10'0,"1"-1"0,0 1 0,0 0 0,7-17 0,1-9 0,-9 31 0,10-44 0,24-65 0,-33 109 0,1 1 0,-1 0 0,1-1 0,0 1 0,0 0 0,0 0 0,1 1 0,0-1 0,-1 1 0,1-1 0,1 1 0,-1 0 0,0 1 0,5-3 0,11-5 0,1 2 0,22-8 0,24-9 0,-27 5-455,0 2 0,68-19 0,-90 32-6371</inkml:trace>
   <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="1700.57">2078 723 24575,'-9'0'0,"0"1"0,0 1 0,0 0 0,0 0 0,0 0 0,0 1 0,1 1 0,-1-1 0,1 1 0,0 1 0,0-1 0,0 1 0,1 1 0,0 0 0,0 0 0,0 0 0,-9 12 0,5-5 0,1 0 0,0 0 0,1 1 0,1 1 0,0 0 0,1 0 0,1 0 0,-8 28 0,4-7 0,2-4 0,-8 48 0,15-72 0,1 0 0,-1 0 0,1 0 0,1 1 0,-1-1 0,1 0 0,1 0 0,0 0 0,0 0 0,0 0 0,5 8 0,-4-12 0,0-1 0,0 0 0,0 1 0,0-2 0,1 1 0,-1 0 0,1 0 0,0-1 0,-1 0 0,1 0 0,0 0 0,1 0 0,-1-1 0,0 0 0,0 1 0,1-1 0,-1-1 0,1 1 0,-1-1 0,9 0 0,13 1 0,0-1 0,31-5 0,-50 4 0,7 0 0,1-2 0,-1 1 0,0-2 0,0 0 0,0 0 0,0-2 0,-1 1 0,0-2 0,0 0 0,0 0 0,-1-1 0,16-13 0,-26 18-151,1 1-1,-1-1 0,0 0 0,0 0 1,0 0-1,-1 0 0,1 0 1,1-6-1,2-9-6674</inkml:trace>
 </inkml:ink>
 </file>

</xml_diff>